<commit_message>
chore(ai-sec): weekly snapshot 2026-05-18
</commit_message>
<xml_diff>
--- a/ai-security-startup-tracker/AI_Security_Startup_Tracker.xlsx
+++ b/ai-security-startup-tracker/AI_Security_Startup_Tracker.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup Ideas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Log" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People &amp; Thought Leaders" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Companies'!$A$1:$L$91</definedName>
@@ -30,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -100,8 +101,11 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +116,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
+        <bgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +159,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -207,6 +217,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -792,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="9" min="1" max="1"/>
@@ -7842,6 +7858,62 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Helmet Security</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Washington DC, USA</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Fred Kneip (CEO, ex-CyberGRX), Kaushik Shanadi (CTO)</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Agentic AI security / MCP security</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>9</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>SYN Ventures, WhiteRabbit Ventures</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Agentic AI security platform — finds, manages, and monitors MCP (Model Context Protocol) servers and connections. Integrates with existing EDR for installation-free visibility into agent communication.</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Emerged from stealth Dec 2025 with $9M seed. Founder Kneip previously built CyberGRX (acquired by ProcessUnity/Marlin). One of the earliest MCP-focused security platforms.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L91"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -7856,7 +7928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="9" min="1" max="1"/>
@@ -9788,6 +9860,46 @@
       <c r="H49" s="9" t="inlineStr">
         <is>
           <t>Backfill — historical round we missed when adding Corgea in methodology fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Helmet Security</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>9</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SYN Ventures, WhiteRabbit Ventures</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Agentic AI security / MCP security</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Stealth emergence; product = MCP server discovery + governance integrated with EDR.</t>
         </is>
       </c>
     </row>
@@ -13928,4 +14040,886 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" style="10" min="1" max="1"/>
+    <col width="22" customWidth="1" style="10" min="2" max="2"/>
+    <col width="30" customWidth="1" style="10" min="3" max="3"/>
+    <col width="26" customWidth="1" style="10" min="4" max="4"/>
+    <col width="36" customWidth="1" style="10" min="5" max="5"/>
+    <col width="36" customWidth="1" style="10" min="6" max="6"/>
+    <col width="16" customWidth="1" style="10" min="7" max="7"/>
+    <col width="20" customWidth="1" style="10" min="8" max="8"/>
+    <col width="50" customWidth="1" style="10" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Affiliation (current)</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Focus areas</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Public output</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Twitter/X</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Joshua Saxe</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Twelve (founder); ex-Meta, ex-Sophos</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Founder / AI security researcher</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>ML for security, GenAI defense, adversarial ML</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>Twitter threads; conference talks; ex-Meta AI security org leadership</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>@joshua_saxe</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>joshuasaxe</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>One of the most-cited voices on practical ML-for-security. Recently focused on agent security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Florian Tramèr</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>Professor / researcher</t>
+        </is>
+      </c>
+      <c r="E3" s="21" t="inlineStr">
+        <is>
+          <t>Adversarial ML, agent security, prompt injection, model extraction</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>Academic papers (NDSS, USENIX, ICML); blog</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="inlineStr">
+        <is>
+          <t>@florian_tramer</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="inlineStr">
+        <is>
+          <t>florian-tramer</t>
+        </is>
+      </c>
+      <c r="I3" s="21" t="inlineStr">
+        <is>
+          <t>Co-author of seminal adversarial ML papers; recent work on tool-call attacks against LLM agents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Nicholas Carlini</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Anthropic (researcher); ex-Google Brain</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Research scientist</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Adversarial attacks on ML, privacy attacks, robustness</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Academic papers; personal blog (nicholas.carlini.com)</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>@nicholascarlini</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>nicholascarlini</t>
+        </is>
+      </c>
+      <c r="I4" s="21" t="inlineStr">
+        <is>
+          <t>Prolific in adversarial ML; many memorable demonstrations of attacks on production models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Peter Garraghan</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Mindgard (CEO/founder); Lancaster University</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Founder / professor</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>AI red teaming, automated adversarial evaluation</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Academic papers; Mindgard blog; conference talks</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>@peter_garraghan</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>petergarraghan</t>
+        </is>
+      </c>
+      <c r="I5" s="21" t="inlineStr">
+        <is>
+          <t>Bridges academic AI security research with commercial AI red-teaming products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Yi Zeng</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Virginia Tech</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Assistant professor / researcher</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>AI safety, jailbreak robustness, alignment evaluation</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Academic papers; Twitter analysis threads</t>
+        </is>
+      </c>
+      <c r="G6" s="21" t="inlineStr">
+        <is>
+          <t>@YiZeng16</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>yi-zeng-research</t>
+        </is>
+      </c>
+      <c r="I6" s="21" t="inlineStr">
+        <is>
+          <t>Often surfaces new jailbreak categories shortly after they appear in the wild.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Itamar Golan</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Prompt Security (CEO/co-founder)</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Founder / commentator</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>GenAI runtime security, LLM firewall, prompt injection defense</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Blog posts; LinkedIn analysis; podcast appearances</t>
+        </is>
+      </c>
+      <c r="G7" s="21" t="inlineStr">
+        <is>
+          <t>@itamar_golan</t>
+        </is>
+      </c>
+      <c r="H7" s="21" t="inlineStr">
+        <is>
+          <t>itamargolan</t>
+        </is>
+      </c>
+      <c r="I7" s="21" t="inlineStr">
+        <is>
+          <t>Influential in shaping the 'GenAI firewall' product category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Edward Wu</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Dropzone AI (CEO/founder)</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>AI-SOC, autonomous alert triage</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Conference talks; LinkedIn posts; technical blog</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="inlineStr">
+        <is>
+          <t>@_edwardwu</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>edwardwu</t>
+        </is>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
+          <t>Defining the AI-SOC category; ex-ExtraHop AI lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Niv Braun</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Noma Security (CEO/founder)</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>AI lifecycle security, agentic AI runtime controls, non-human identity</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>Conference talks; LinkedIn posts; podcast appearances</t>
+        </is>
+      </c>
+      <c r="G9" s="21" t="inlineStr">
+        <is>
+          <t>@nivbraun</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
+        <is>
+          <t>nivbraun</t>
+        </is>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>Pushes the framing of 'AI lifecycle' as a security category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Fred Kneip</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Helmet Security (CEO/co-founder); ex-CyberGRX (founder)</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Founder / serial entrepreneur</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>Agentic AI security, MCP governance, third-party cyber risk (prior)</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Conference talks; LinkedIn posts; CyberGRX legacy</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>fredkneip</t>
+        </is>
+      </c>
+      <c r="I10" s="21" t="inlineStr">
+        <is>
+          <t>Built CyberGRX ($100M+ raised, acquired by ProcessUnity); now leading Helmet's MCP-focused agentic AI security platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Kaushik Shanadi</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>Helmet Security (CTO/co-founder)</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Founder / CTO</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>Agentic AI security, MCP server discovery and policy enforcement, EDR integration</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>Helmet engineering posts; LinkedIn</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>kaushikshanadi</t>
+        </is>
+      </c>
+      <c r="I11" s="21" t="inlineStr">
+        <is>
+          <t>Helmet co-founder; technical architect behind the platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Jason Clinton</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>Anthropic (CISO)</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Security leadership</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Frontier model security, agent security, applied security at AI labs</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Conference talks; LinkedIn posts; interviews</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>jasonclinton</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
+          <t>Voice for how frontier AI labs think about security internally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Daniel Bohannon</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>SpecterOps; ex-Mandiant</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>Researcher / red team</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Offensive security automation, obfuscation, attacker tradecraft</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>Conference talks (DefCon, Bsides); GitHub tooling; Twitter</t>
+        </is>
+      </c>
+      <c r="G13" s="21" t="inlineStr">
+        <is>
+          <t>@danielhbohannon</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
+        <is>
+          <t>danielbohannon</t>
+        </is>
+      </c>
+      <c r="I13" s="21" t="inlineStr">
+        <is>
+          <t>Influential on offensive security tooling; relevant as AI-aided offense matures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Daniel Miessler</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>Unsupervised Learning (newsletter/podcast)</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Analyst / commentator</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>AI x security intersection, threat trends, practitioner POV</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>Unsupervised Learning newsletter (~100k+ subscribers); podcast</t>
+        </is>
+      </c>
+      <c r="G14" s="21" t="inlineStr">
+        <is>
+          <t>@DanielMiessler</t>
+        </is>
+      </c>
+      <c r="H14" s="21" t="inlineStr">
+        <is>
+          <t>danielmiessler</t>
+        </is>
+      </c>
+      <c r="I14" s="21" t="inlineStr">
+        <is>
+          <t>Probably the most-read newsletter at the AI x security intersection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Ross Haleliuk</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>Venture in Security (newsletter); LimaCharlie</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>Analyst / writer / operator</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>Cybersecurity market analysis, GTM, founder commentary</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>Venture in Security newsletter; LinkedIn posts; book ('Cyber for Builders')</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>@RossHaleliuk</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
+        <is>
+          <t>rosshaleliuk</t>
+        </is>
+      </c>
+      <c r="I15" s="21" t="inlineStr">
+        <is>
+          <t>Required reading for cybersecurity founders and investors; cross-pollinates AI security topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Rich Mogull</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Securosis (founder); Defense Storm</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Cloud security, security architecture, vendor analysis</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Securosis blog; speaking; published research</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="inlineStr">
+        <is>
+          <t>@rmogull</t>
+        </is>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>rmogull</t>
+        </is>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
+        <is>
+          <t>Veteran analyst whose vendor takedowns are widely respected; growing AI security coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>HD Moore</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>runZero (CEO/founder); creator of Metasploit</t>
+        </is>
+      </c>
+      <c r="D17" s="21" t="inlineStr">
+        <is>
+          <t>Founder / pioneer</t>
+        </is>
+      </c>
+      <c r="E17" s="21" t="inlineStr">
+        <is>
+          <t>Asset discovery, attack surface, security research</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>runZero blog; conference talks; LinkedIn</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>@hdmoore</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
+        <is>
+          <t>hdmoore</t>
+        </is>
+      </c>
+      <c r="I17" s="21" t="inlineStr">
+        <is>
+          <t>Iconic security figure; runZero is increasingly relevant for AI agent inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Bruce Schneier</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Harvard Kennedy School; Schneier on Security blog</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Cryptographer / public intellectual</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Security and society, AI governance, policy</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Schneier on Security blog; books; columns</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="inlineStr">
+        <is>
+          <t>@schneierblog</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>bruceschneier</t>
+        </is>
+      </c>
+      <c r="I18" s="21" t="inlineStr">
+        <is>
+          <t>Long-form thinking on the societal/policy edges of AI security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>Helen Toner</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>CSET (Georgetown); ex-OpenAI board</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Policy researcher</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>AI governance, frontier risk, national security policy</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>CSET reports; congressional testimony; podcast</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>@hlntnr</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>helen-toner</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
+          <t>Influential on Washington's view of AI risk and governance.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>